<commit_message>
kanban: S00 done、S01〜S04 を In Progress へ
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/kanban.xlsx
+++ b/docs/kanban.xlsx
@@ -78,7 +78,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -98,6 +98,12 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -465,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -477,98 +483,94 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Backlog (8)</t>
+          <t>Backlog (4)</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>In Progress (0)</t>
+          <t>In Progress (4)</t>
         </is>
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>Review(Qodo) (1)</t>
+          <t>Review(Qodo) (0)</t>
         </is>
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
-          <t>Done (0)</t>
+          <t>Done (1)</t>
         </is>
       </c>
       <c r="F1" s="5" t="inlineStr">
         <is>
-          <t>updated 2026-08-29 15:42</t>
+          <t>updated 2026-08-29 15:43</t>
         </is>
       </c>
     </row>
     <row r="2" ht="58" customHeight="1">
       <c r="A2" s="6" t="inlineStr">
         <is>
+          <t>S05  召喚 `aishow summon`(TrueForge API・承認 → cast)
+ · 2026-08-29 15:42</t>
+        </is>
+      </c>
+      <c r="B2" s="10" t="inlineStr">
+        <is>
           <t>S01  ハーネス(TrueForge + OpenAI + Bright Data MCP + 呪文)
- · 2026-08-29 15:42</t>
-        </is>
-      </c>
-      <c r="C2" s="8" t="inlineStr">
+agent · 2026-08-29 15:43
+担当官: TrueForge API 調査 + 呪文精緻化</t>
+        </is>
+      </c>
+      <c r="D2" s="9" t="inlineStr">
         <is>
           <t>S00  骨組み(Package / .gitignore / Qodo / 発注書 / kanban)
-fable · 2026-08-29 15:42
-ビルド・テスト OK、コミット待ち</t>
+fable · 2026-08-29 15:43
+commit 5ce3888(push は主権者承認待ち)</t>
         </is>
       </c>
     </row>
     <row r="3" ht="58" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
+          <t>S06  常駐 `Aishow.app`(メニューバー・ホットキー・承認 UI)
+ · 2026-08-29 15:42</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
           <t>S02  索敵・特定 `aishow scan`(ContextPack / detect)
- · 2026-08-29 15:42</t>
+agent · 2026-08-29 15:43
+担当官: worktree step-02</t>
         </is>
       </c>
     </row>
     <row r="4" ht="58" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
+          <t>D01  デモ動画(3 分)・README 仕上げ
+ · 2026-08-29 15:42</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
           <t>S03  発動 `aishow cast`(貼り付け・クリップボード復元)
- · 2026-08-29 15:42</t>
+agent · 2026-08-29 15:43
+担当官: worktree step-03</t>
         </is>
       </c>
     </row>
     <row r="5" ht="58" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>S04  詠唱 `aishow chant`(録音 → OpenAI STT)
- · 2026-08-29 15:42</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="58" customHeight="1">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>S05  召喚 `aishow summon`(TrueForge API・承認 → cast)
- · 2026-08-29 15:42</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="58" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>S06  常駐 `Aishow.app`(メニューバー・ホットキー・承認 UI)
- · 2026-08-29 15:42</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="58" customHeight="1">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>D01  デモ動画(3 分)・README 仕上げ
- · 2026-08-29 15:42</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="58" customHeight="1">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
           <t>D02  提出フォーム(Q8–Q19)
  · 2026-08-29 15:42</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>S04  詠唱 `aishow chant`(録音 → OpenAI STT)
+agent · 2026-08-29 15:43
+担当官: worktree step-04</t>
         </is>
       </c>
     </row>
@@ -650,7 +652,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>done</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -660,12 +662,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-08-29 15:42</t>
+          <t>2026-08-29 15:43</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>ビルド・テスト OK、コミット待ち</t>
+          <t>commit 5ce3888(push は主権者承認待ち)</t>
         </is>
       </c>
     </row>
@@ -687,12 +689,22 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>backlog</t>
+          <t>doing</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>agent</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-08-29 15:42</t>
+          <t>2026-08-29 15:43</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>担当官: TrueForge API 調査 + 呪文精緻化</t>
         </is>
       </c>
     </row>
@@ -714,12 +726,22 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>backlog</t>
+          <t>doing</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>agent</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-08-29 15:42</t>
+          <t>2026-08-29 15:43</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>担当官: worktree step-02</t>
         </is>
       </c>
     </row>
@@ -741,12 +763,22 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>backlog</t>
+          <t>doing</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>agent</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-08-29 15:42</t>
+          <t>2026-08-29 15:43</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>担当官: worktree step-03</t>
         </is>
       </c>
     </row>
@@ -768,12 +800,22 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>backlog</t>
+          <t>doing</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>agent</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-08-29 15:42</t>
+          <t>2026-08-29 15:43</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>担当官: worktree step-04</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
kanban: S02〜S04 を Review へ
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/kanban.xlsx
+++ b/docs/kanban.xlsx
@@ -488,12 +488,12 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>In Progress (4)</t>
+          <t>In Progress (1)</t>
         </is>
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>Review(Qodo) (0)</t>
+          <t>Review(Qodo) (3)</t>
         </is>
       </c>
       <c r="D1" s="4" t="inlineStr">
@@ -503,7 +503,7 @@
       </c>
       <c r="F1" s="5" t="inlineStr">
         <is>
-          <t>updated 2026-08-29 15:43</t>
+          <t>updated 2026-08-29 15:52</t>
         </is>
       </c>
     </row>
@@ -521,6 +521,13 @@
 担当官: TrueForge API 調査 + 呪文精緻化</t>
         </is>
       </c>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t>S02  索敵・特定 `aishow scan`(ContextPack / detect)
+agent · 2026-08-29 15:51
+実装完了・12 tests 通過。PR 待ち</t>
+        </is>
+      </c>
       <c r="D2" s="9" t="inlineStr">
         <is>
           <t>S00  骨組み(Package / .gitignore / Qodo / 発注書 / kanban)
@@ -536,11 +543,11 @@
  · 2026-08-29 15:42</t>
         </is>
       </c>
-      <c r="B3" s="10" t="inlineStr">
-        <is>
-          <t>S02  索敵・特定 `aishow scan`(ContextPack / detect)
-agent · 2026-08-29 15:43
-担当官: worktree step-02</t>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>S03  発動 `aishow cast`(貼り付け・クリップボード復元)
+agent · 2026-08-29 15:51
+実装完了・TextEdit 実機 OK。PR 待ち</t>
         </is>
       </c>
     </row>
@@ -551,11 +558,11 @@
  · 2026-08-29 15:42</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
-        <is>
-          <t>S03  発動 `aishow cast`(貼り付け・クリップボード復元)
-agent · 2026-08-29 15:43
-担当官: worktree step-03</t>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>S04  詠唱 `aishow chant`(録音 → OpenAI STT)
+agent · 2026-08-29 15:52
+実装完了。OPENAI_API_KEY が 401 のため実 STT は未検証 → 主権者がキー更新</t>
         </is>
       </c>
     </row>
@@ -564,13 +571,6 @@
         <is>
           <t>D02  提出フォーム(Q8–Q19)
  · 2026-08-29 15:42</t>
-        </is>
-      </c>
-      <c r="B5" s="10" t="inlineStr">
-        <is>
-          <t>S04  詠唱 `aishow chant`(録音 → OpenAI STT)
-agent · 2026-08-29 15:43
-担当官: worktree step-04</t>
         </is>
       </c>
     </row>
@@ -726,7 +726,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>doing</t>
+          <t>review</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -736,12 +736,12 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-08-29 15:43</t>
+          <t>2026-08-29 15:51</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>担当官: worktree step-02</t>
+          <t>実装完了・12 tests 通過。PR 待ち</t>
         </is>
       </c>
     </row>
@@ -763,7 +763,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>doing</t>
+          <t>review</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -773,12 +773,12 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-08-29 15:43</t>
+          <t>2026-08-29 15:51</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>担当官: worktree step-03</t>
+          <t>実装完了・TextEdit 実機 OK。PR 待ち</t>
         </is>
       </c>
     </row>
@@ -800,7 +800,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>doing</t>
+          <t>review</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -810,12 +810,12 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-08-29 15:43</t>
+          <t>2026-08-29 15:52</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>担当官: worktree step-04</t>
+          <t>実装完了。OPENAI_API_KEY が 401 のため実 STT は未検証 → 主権者がキー更新</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
kanban: S01 Review、S05 In Progress
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/kanban.xlsx
+++ b/docs/kanban.xlsx
@@ -483,7 +483,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Backlog (4)</t>
+          <t>Backlog (3)</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
@@ -493,7 +493,7 @@
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>Review(Qodo) (3)</t>
+          <t>Review(Qodo) (4)</t>
         </is>
       </c>
       <c r="D1" s="4" t="inlineStr">
@@ -503,47 +503,62 @@
       </c>
       <c r="F1" s="5" t="inlineStr">
         <is>
-          <t>updated 2026-08-29 15:52</t>
+          <t>updated 2026-08-29 15:59</t>
         </is>
       </c>
     </row>
     <row r="2" ht="58" customHeight="1">
       <c r="A2" s="6" t="inlineStr">
         <is>
+          <t>S06  常駐 `Aishow.app`(メニューバー・ホットキー・承認 UI)
+ · 2026-08-29 15:42</t>
+        </is>
+      </c>
+      <c r="B2" s="10" t="inlineStr">
+        <is>
           <t>S05  召喚 `aishow summon`(TrueForge API・承認 → cast)
+agent · 2026-08-29 15:59
+担当官: worktree step-05(承認は CLI 側)</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t>S01  ハーネス(TrueForge + OpenAI + Bright Data MCP + 呪文)
+agent · 2026-08-29 15:59
+API 調査完了(trueforge-api.md)。Bright Data 実接続・collector は持ち越し</t>
+        </is>
+      </c>
+      <c r="D2" s="9" t="inlineStr">
+        <is>
+          <t>S00  骨組み(Package / .gitignore / Qodo / 発注書 / kanban)
+fable · 2026-08-29 15:43
+commit 5ce3888(push は主権者承認待ち)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="58" customHeight="1">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>D01  デモ動画(3 分)・README 仕上げ
  · 2026-08-29 15:42</t>
         </is>
       </c>
-      <c r="B2" s="10" t="inlineStr">
-        <is>
-          <t>S01  ハーネス(TrueForge + OpenAI + Bright Data MCP + 呪文)
-agent · 2026-08-29 15:43
-担当官: TrueForge API 調査 + 呪文精緻化</t>
-        </is>
-      </c>
-      <c r="C2" s="8" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>S02  索敵・特定 `aishow scan`(ContextPack / detect)
 agent · 2026-08-29 15:51
 実装完了・12 tests 通過。PR 待ち</t>
         </is>
       </c>
-      <c r="D2" s="9" t="inlineStr">
-        <is>
-          <t>S00  骨組み(Package / .gitignore / Qodo / 発注書 / kanban)
-fable · 2026-08-29 15:43
-commit 5ce3888(push は主権者承認待ち)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="58" customHeight="1">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>S06  常駐 `Aishow.app`(メニューバー・ホットキー・承認 UI)
+    </row>
+    <row r="4" ht="58" customHeight="1">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>D02  提出フォーム(Q8–Q19)
  · 2026-08-29 15:42</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C4" s="8" t="inlineStr">
         <is>
           <t>S03  発動 `aishow cast`(貼り付け・クリップボード復元)
 agent · 2026-08-29 15:51
@@ -551,26 +566,12 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="58" customHeight="1">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>D01  デモ動画(3 分)・README 仕上げ
- · 2026-08-29 15:42</t>
-        </is>
-      </c>
-      <c r="C4" s="8" t="inlineStr">
+    <row r="5" ht="58" customHeight="1">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>S04  詠唱 `aishow chant`(録音 → OpenAI STT)
 agent · 2026-08-29 15:52
 実装完了。OPENAI_API_KEY が 401 のため実 STT は未検証 → 主権者がキー更新</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="58" customHeight="1">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>D02  提出フォーム(Q8–Q19)
- · 2026-08-29 15:42</t>
         </is>
       </c>
     </row>
@@ -689,7 +690,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>doing</t>
+          <t>review</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -699,12 +700,12 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-08-29 15:43</t>
+          <t>2026-08-29 15:59</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>担当官: TrueForge API 調査 + 呪文精緻化</t>
+          <t>API 調査完了(trueforge-api.md)。Bright Data 実接続・collector は持ち越し</t>
         </is>
       </c>
     </row>
@@ -837,12 +838,22 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>backlog</t>
+          <t>doing</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>agent</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-08-29 15:42</t>
+          <t>2026-08-29 15:59</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>担当官: worktree step-05(承認は CLI 側)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
kanban: S06 In Progress
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/kanban.xlsx
+++ b/docs/kanban.xlsx
@@ -483,12 +483,12 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Backlog (3)</t>
+          <t>Backlog (2)</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>In Progress (1)</t>
+          <t>In Progress (2)</t>
         </is>
       </c>
       <c r="C1" s="3" t="inlineStr">
@@ -503,14 +503,14 @@
       </c>
       <c r="F1" s="5" t="inlineStr">
         <is>
-          <t>updated 2026-08-29 15:59</t>
+          <t>updated 2026-08-29 16:00</t>
         </is>
       </c>
     </row>
     <row r="2" ht="58" customHeight="1">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>S06  常駐 `Aishow.app`(メニューバー・ホットキー・承認 UI)
+          <t>D01  デモ動画(3 分)・README 仕上げ
  · 2026-08-29 15:42</t>
         </is>
       </c>
@@ -539,8 +539,15 @@
     <row r="3" ht="58" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>D01  デモ動画(3 分)・README 仕上げ
+          <t>D02  提出フォーム(Q8–Q19)
  · 2026-08-29 15:42</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>S06  常駐 `Aishow.app`(メニューバー・ホットキー・承認 UI)
+agent · 2026-08-29 16:00
+担当官: worktree step-06(App 殻を先行、summon 結線は S05 後)</t>
         </is>
       </c>
       <c r="C3" s="8" t="inlineStr">
@@ -552,12 +559,6 @@
       </c>
     </row>
     <row r="4" ht="58" customHeight="1">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>D02  提出フォーム(Q8–Q19)
- · 2026-08-29 15:42</t>
-        </is>
-      </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
           <t>S03  発動 `aishow cast`(貼り付け・クリップボード復元)
@@ -875,12 +876,22 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>backlog</t>
+          <t>doing</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>agent</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-08-29 15:42</t>
+          <t>2026-08-29 16:00</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>担当官: worktree step-06(App 殻を先行、summon 結線は S05 後)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
kanban: S05 Review、S06 結線中
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/kanban.xlsx
+++ b/docs/kanban.xlsx
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -488,12 +488,12 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>In Progress (1)</t>
+          <t>In Progress (0)</t>
         </is>
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>Review(Qodo) (5)</t>
+          <t>Review(Qodo) (6)</t>
         </is>
       </c>
       <c r="D1" s="4" t="inlineStr">
@@ -503,7 +503,7 @@
       </c>
       <c r="F1" s="5" t="inlineStr">
         <is>
-          <t>updated 2026-08-29 16:06</t>
+          <t>updated 2026-08-29 16:08</t>
         </is>
       </c>
     </row>
@@ -512,13 +512,6 @@
         <is>
           <t>D01  デモ動画(3 分)・README 仕上げ
  · 2026-08-29 15:42</t>
-        </is>
-      </c>
-      <c r="B2" s="10" t="inlineStr">
-        <is>
-          <t>S05  召喚 `aishow summon`(TrueForge API・承認 → cast)
-agent · 2026-08-29 15:59
-担当官: worktree step-05(承認は CLI 側)</t>
         </is>
       </c>
       <c r="C2" s="8" t="inlineStr">
@@ -572,9 +565,18 @@
     <row r="6" ht="58" customHeight="1">
       <c r="C6" s="8" t="inlineStr">
         <is>
+          <t>S05  召喚 `aishow summon`(TrueForge API・承認 → cast)
+agent · 2026-08-29 16:08
+実装完了(TrueForge API 実機疎通)。OPENAI キー無効のため生成は未検証</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="58" customHeight="1">
+      <c r="C7" s="8" t="inlineStr">
+        <is>
           <t>S06  常駐 `Aishow.app`(メニューバー・ホットキー・承認 UI)
-agent · 2026-08-29 16:06
-App 殻完了(make app OK、常駐確認)。summon 結線は S05 後</t>
+agent · 2026-08-29 16:08
+S05 と結線中(worktree step-07)</t>
         </is>
       </c>
     </row>
@@ -841,7 +843,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>doing</t>
+          <t>review</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -851,12 +853,12 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-08-29 15:59</t>
+          <t>2026-08-29 16:08</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>担当官: worktree step-05(承認は CLI 側)</t>
+          <t>実装完了(TrueForge API 実機疎通)。OPENAI キー無効のため生成は未検証</t>
         </is>
       </c>
     </row>
@@ -888,12 +890,12 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-08-29 16:06</t>
+          <t>2026-08-29 16:08</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>App 殻完了(make app OK、常駐確認)。summon 結線は S05 後</t>
+          <t>S05 と結線中(worktree step-07)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
kanban: PR #1〜#6 を記録
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/kanban.xlsx
+++ b/docs/kanban.xlsx
@@ -503,7 +503,7 @@
       </c>
       <c r="F1" s="5" t="inlineStr">
         <is>
-          <t>updated 2026-08-29 16:08</t>
+          <t>updated 2026-08-29 16:10</t>
         </is>
       </c>
     </row>
@@ -517,8 +517,8 @@
       <c r="C2" s="8" t="inlineStr">
         <is>
           <t>S01  ハーネス(TrueForge + OpenAI + Bright Data MCP + 呪文)
-agent · 2026-08-29 15:59
-API 調査完了(trueforge-api.md)。Bright Data 実接続・collector は持ち越し</t>
+agent · 2026-08-29 16:10
+PR #1 https://github.com/yossitv/aishow/pull/1(Qodo 待ち)</t>
         </is>
       </c>
       <c r="D2" s="9" t="inlineStr">
@@ -539,8 +539,8 @@
       <c r="C3" s="8" t="inlineStr">
         <is>
           <t>S02  索敵・特定 `aishow scan`(ContextPack / detect)
-agent · 2026-08-29 15:51
-実装完了・12 tests 通過。PR 待ち</t>
+agent · 2026-08-29 16:10
+PR #2 https://github.com/yossitv/aishow/pull/2(Qodo 待ち)</t>
         </is>
       </c>
     </row>
@@ -548,8 +548,8 @@
       <c r="C4" s="8" t="inlineStr">
         <is>
           <t>S03  発動 `aishow cast`(貼り付け・クリップボード復元)
-agent · 2026-08-29 15:51
-実装完了・TextEdit 実機 OK。PR 待ち</t>
+agent · 2026-08-29 16:10
+PR #3 https://github.com/yossitv/aishow/pull/3(Qodo 待ち)</t>
         </is>
       </c>
     </row>
@@ -557,8 +557,8 @@
       <c r="C5" s="8" t="inlineStr">
         <is>
           <t>S04  詠唱 `aishow chant`(録音 → OpenAI STT)
-agent · 2026-08-29 15:52
-実装完了。OPENAI_API_KEY が 401 のため実 STT は未検証 → 主権者がキー更新</t>
+agent · 2026-08-29 16:10
+PR #4 https://github.com/yossitv/aishow/pull/4(Qodo 待ち)</t>
         </is>
       </c>
     </row>
@@ -566,8 +566,8 @@
       <c r="C6" s="8" t="inlineStr">
         <is>
           <t>S05  召喚 `aishow summon`(TrueForge API・承認 → cast)
-agent · 2026-08-29 16:08
-実装完了(TrueForge API 実機疎通)。OPENAI キー無効のため生成は未検証</t>
+agent · 2026-08-29 16:10
+PR #5 https://github.com/yossitv/aishow/pull/5(Qodo 待ち)</t>
         </is>
       </c>
     </row>
@@ -575,8 +575,8 @@
       <c r="C7" s="8" t="inlineStr">
         <is>
           <t>S06  常駐 `Aishow.app`(メニューバー・ホットキー・承認 UI)
-agent · 2026-08-29 16:08
-S05 と結線中(worktree step-07)</t>
+agent · 2026-08-29 16:10
+PR #6 https://github.com/yossitv/aishow/pull/6(Qodo 待ち)</t>
         </is>
       </c>
     </row>
@@ -705,12 +705,12 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-08-29 15:59</t>
+          <t>2026-08-29 16:10</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>API 調査完了(trueforge-api.md)。Bright Data 実接続・collector は持ち越し</t>
+          <t>PR #1 https://github.com/yossitv/aishow/pull/1(Qodo 待ち)</t>
         </is>
       </c>
     </row>
@@ -742,12 +742,12 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-08-29 15:51</t>
+          <t>2026-08-29 16:10</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>実装完了・12 tests 通過。PR 待ち</t>
+          <t>PR #2 https://github.com/yossitv/aishow/pull/2(Qodo 待ち)</t>
         </is>
       </c>
     </row>
@@ -779,12 +779,12 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-08-29 15:51</t>
+          <t>2026-08-29 16:10</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>実装完了・TextEdit 実機 OK。PR 待ち</t>
+          <t>PR #3 https://github.com/yossitv/aishow/pull/3(Qodo 待ち)</t>
         </is>
       </c>
     </row>
@@ -816,12 +816,12 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-08-29 15:52</t>
+          <t>2026-08-29 16:10</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>実装完了。OPENAI_API_KEY が 401 のため実 STT は未検証 → 主権者がキー更新</t>
+          <t>PR #4 https://github.com/yossitv/aishow/pull/4(Qodo 待ち)</t>
         </is>
       </c>
     </row>
@@ -853,12 +853,12 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-08-29 16:08</t>
+          <t>2026-08-29 16:10</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>実装完了(TrueForge API 実機疎通)。OPENAI キー無効のため生成は未検証</t>
+          <t>PR #5 https://github.com/yossitv/aishow/pull/5(Qodo 待ち)</t>
         </is>
       </c>
     </row>
@@ -890,12 +890,12 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-08-29 16:08</t>
+          <t>2026-08-29 16:10</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>S05 と結線中(worktree step-07)</t>
+          <t>PR #6 https://github.com/yossitv/aishow/pull/6(Qodo 待ち)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
kanban: S01〜S04 Done(PR マージ)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/kanban.xlsx
+++ b/docs/kanban.xlsx
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -493,17 +493,17 @@
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>Review(Qodo) (6)</t>
+          <t>Review(Qodo) (2)</t>
         </is>
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
-          <t>Done (1)</t>
+          <t>Done (5)</t>
         </is>
       </c>
       <c r="F1" s="5" t="inlineStr">
         <is>
-          <t>updated 2026-08-29 16:14</t>
+          <t>updated 2026-08-29 16:28</t>
         </is>
       </c>
     </row>
@@ -516,9 +516,9 @@
       </c>
       <c r="C2" s="8" t="inlineStr">
         <is>
-          <t>S01  ハーネス(TrueForge + OpenAI + Bright Data MCP + 呪文)
-agent · 2026-08-29 16:14
-PR #1 Qodo レビュー済(High あり → step-07-wire で修正中)</t>
+          <t>S05  召喚 `aishow summon`(TrueForge API・承認 → cast)
+agent · 2026-08-29 16:28
+PR #5 は main と衝突 → PR #7(step-07-wire)で置換</t>
         </is>
       </c>
       <c r="D2" s="9" t="inlineStr">
@@ -538,45 +538,43 @@
       </c>
       <c r="C3" s="8" t="inlineStr">
         <is>
+          <t>S06  常駐 `Aishow.app`(メニューバー・ホットキー・承認 UI)
+agent · 2026-08-29 16:28
+PR #6 は main と衝突 → PR #7(step-07-wire)で置換</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>S01  ハーネス(TrueForge + OpenAI + Bright Data MCP + 呪文)
+agent · 2026-08-29 16:28
+PR #1 マージ済(Qodo High は PR #7 で対応)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="58" customHeight="1">
+      <c r="D4" s="9" t="inlineStr">
+        <is>
           <t>S02  索敵・特定 `aishow scan`(ContextPack / detect)
-agent · 2026-08-29 16:14
-PR #2 Qodo レビュー済(High あり → step-07-wire で修正中)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="58" customHeight="1">
-      <c r="C4" s="8" t="inlineStr">
+agent · 2026-08-29 16:28
+PR #2 マージ済(Qodo High は PR #7 で対応)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="58" customHeight="1">
+      <c r="D5" s="9" t="inlineStr">
         <is>
           <t>S03  発動 `aishow cast`(貼り付け・クリップボード復元)
-agent · 2026-08-29 16:14
-PR #3 Qodo レビュー済(High あり → step-07-wire で修正中)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="58" customHeight="1">
-      <c r="C5" s="8" t="inlineStr">
+agent · 2026-08-29 16:28
+PR #3 マージ済(Qodo High は PR #7 で対応)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="58" customHeight="1">
+      <c r="D6" s="9" t="inlineStr">
         <is>
           <t>S04  詠唱 `aishow chant`(録音 → OpenAI STT)
-agent · 2026-08-29 16:14
-PR #4 Qodo レビュー済(High あり → step-07-wire で修正中)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="58" customHeight="1">
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>S05  召喚 `aishow summon`(TrueForge API・承認 → cast)
-agent · 2026-08-29 16:14
-PR #5 Qodo レビュー済(High あり → step-07-wire で修正中)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="58" customHeight="1">
-      <c r="C7" s="8" t="inlineStr">
-        <is>
-          <t>S06  常駐 `Aishow.app`(メニューバー・ホットキー・承認 UI)
-agent · 2026-08-29 16:14
-PR #6 Qodo レビュー済(High あり → step-07-wire で修正中)</t>
+agent · 2026-08-29 16:28
+PR #4 マージ済(Qodo High は PR #7 で対応)</t>
         </is>
       </c>
     </row>
@@ -695,7 +693,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>done</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -705,12 +703,12 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-08-29 16:14</t>
+          <t>2026-08-29 16:28</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>PR #1 Qodo レビュー済(High あり → step-07-wire で修正中)</t>
+          <t>PR #1 マージ済(Qodo High は PR #7 で対応)</t>
         </is>
       </c>
     </row>
@@ -732,7 +730,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>done</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -742,12 +740,12 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-08-29 16:14</t>
+          <t>2026-08-29 16:28</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>PR #2 Qodo レビュー済(High あり → step-07-wire で修正中)</t>
+          <t>PR #2 マージ済(Qodo High は PR #7 で対応)</t>
         </is>
       </c>
     </row>
@@ -769,7 +767,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>done</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -779,12 +777,12 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-08-29 16:14</t>
+          <t>2026-08-29 16:28</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>PR #3 Qodo レビュー済(High あり → step-07-wire で修正中)</t>
+          <t>PR #3 マージ済(Qodo High は PR #7 で対応)</t>
         </is>
       </c>
     </row>
@@ -806,7 +804,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>done</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -816,12 +814,12 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-08-29 16:14</t>
+          <t>2026-08-29 16:28</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>PR #4 Qodo レビュー済(High あり → step-07-wire で修正中)</t>
+          <t>PR #4 マージ済(Qodo High は PR #7 で対応)</t>
         </is>
       </c>
     </row>
@@ -853,12 +851,12 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-08-29 16:14</t>
+          <t>2026-08-29 16:28</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>PR #5 Qodo レビュー済(High あり → step-07-wire で修正中)</t>
+          <t>PR #5 は main と衝突 → PR #7(step-07-wire)で置換</t>
         </is>
       </c>
     </row>
@@ -890,12 +888,12 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-08-29 16:14</t>
+          <t>2026-08-29 16:28</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>PR #6 Qodo レビュー済(High あり → step-07-wire で修正中)</t>
+          <t>PR #6 は main と衝突 → PR #7(step-07-wire)で置換</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
kanban: S05/S06 → PR #7
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/kanban.xlsx
+++ b/docs/kanban.xlsx
@@ -503,7 +503,7 @@
       </c>
       <c r="F1" s="5" t="inlineStr">
         <is>
-          <t>updated 2026-08-29 16:28</t>
+          <t>updated 2026-08-29 16:38</t>
         </is>
       </c>
     </row>
@@ -517,8 +517,8 @@
       <c r="C2" s="8" t="inlineStr">
         <is>
           <t>S05  召喚 `aishow summon`(TrueForge API・承認 → cast)
-agent · 2026-08-29 16:28
-PR #5 は main と衝突 → PR #7(step-07-wire)で置換</t>
+agent · 2026-08-29 16:38
+PR #7(結線)で Qodo 待ち</t>
         </is>
       </c>
       <c r="D2" s="9" t="inlineStr">
@@ -539,8 +539,8 @@
       <c r="C3" s="8" t="inlineStr">
         <is>
           <t>S06  常駐 `Aishow.app`(メニューバー・ホットキー・承認 UI)
-agent · 2026-08-29 16:28
-PR #6 は main と衝突 → PR #7(step-07-wire)で置換</t>
+agent · 2026-08-29 16:38
+PR #7(結線)で Qodo 待ち</t>
         </is>
       </c>
       <c r="D3" s="9" t="inlineStr">
@@ -851,12 +851,12 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-08-29 16:28</t>
+          <t>2026-08-29 16:38</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>PR #5 は main と衝突 → PR #7(step-07-wire)で置換</t>
+          <t>PR #7(結線)で Qodo 待ち</t>
         </is>
       </c>
     </row>
@@ -888,12 +888,12 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-08-29 16:28</t>
+          <t>2026-08-29 16:38</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>PR #6 は main と衝突 → PR #7(step-07-wire)で置換</t>
+          <t>PR #7(結線)で Qodo 待ち</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
kanban: S05/S06 Done、D01/D02 を主権者へ
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/kanban.xlsx
+++ b/docs/kanban.xlsx
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -483,42 +483,36 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Backlog (2)</t>
+          <t>Backlog (0)</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>In Progress (0)</t>
+          <t>In Progress (2)</t>
         </is>
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>Review(Qodo) (2)</t>
+          <t>Review(Qodo) (0)</t>
         </is>
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
-          <t>Done (5)</t>
+          <t>Done (7)</t>
         </is>
       </c>
       <c r="F1" s="5" t="inlineStr">
         <is>
-          <t>updated 2026-08-29 16:38</t>
+          <t>updated 2026-08-29 16:48</t>
         </is>
       </c>
     </row>
     <row r="2" ht="58" customHeight="1">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="B2" s="10" t="inlineStr">
         <is>
           <t>D01  デモ動画(3 分)・README 仕上げ
- · 2026-08-29 15:42</t>
-        </is>
-      </c>
-      <c r="C2" s="8" t="inlineStr">
-        <is>
-          <t>S05  召喚 `aishow summon`(TrueForge API・承認 → cast)
-agent · 2026-08-29 16:38
-PR #7(結線)で Qodo 待ち</t>
+主権者 · 2026-08-29 16:47
+主権者: docs/demo.md の台本で撮影(3 分)</t>
         </is>
       </c>
       <c r="D2" s="9" t="inlineStr">
@@ -530,17 +524,11 @@
       </c>
     </row>
     <row r="3" ht="58" customHeight="1">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="B3" s="10" t="inlineStr">
         <is>
           <t>D02  提出フォーム(Q8–Q19)
- · 2026-08-29 15:42</t>
-        </is>
-      </c>
-      <c r="C3" s="8" t="inlineStr">
-        <is>
-          <t>S06  常駐 `Aishow.app`(メニューバー・ホットキー・承認 UI)
-agent · 2026-08-29 16:38
-PR #7(結線)で Qodo 待ち</t>
+主権者 · 2026-08-29 16:48
+下書き済(hackathon/agent_harness_20260829/docs/submission.md)。動画 URL を入れて送信</t>
         </is>
       </c>
       <c r="D3" s="9" t="inlineStr">
@@ -575,6 +563,24 @@
           <t>S04  詠唱 `aishow chant`(録音 → OpenAI STT)
 agent · 2026-08-29 16:28
 PR #4 マージ済(Qodo High は PR #7 で対応)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="58" customHeight="1">
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>S05  召喚 `aishow summon`(TrueForge API・承認 → cast)
+agent · 2026-08-29 16:47
+PR #7 マージ(TrueForge 実機で website_form → Bright Data 14 呼び出し → 提案 確認)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="58" customHeight="1">
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>S06  常駐 `Aishow.app`(メニューバー・ホットキー・承認 UI)
+agent · 2026-08-29 16:47
+PR #7 マージ(make app OK、常駐確認。GUI 通しは主権者が実施)</t>
         </is>
       </c>
     </row>
@@ -841,7 +847,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>done</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -851,12 +857,12 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-08-29 16:38</t>
+          <t>2026-08-29 16:47</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>PR #7(結線)で Qodo 待ち</t>
+          <t>PR #7 マージ(TrueForge 実機で website_form → Bright Data 14 呼び出し → 提案 確認)</t>
         </is>
       </c>
     </row>
@@ -878,7 +884,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>done</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -888,12 +894,12 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-08-29 16:38</t>
+          <t>2026-08-29 16:47</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>PR #7(結線)で Qodo 待ち</t>
+          <t>PR #7 マージ(make app OK、常駐確認。GUI 通しは主権者が実施)</t>
         </is>
       </c>
     </row>
@@ -915,12 +921,22 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>backlog</t>
+          <t>doing</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>主権者</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-08-29 15:42</t>
+          <t>2026-08-29 16:47</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>主権者: docs/demo.md の台本で撮影(3 分)</t>
         </is>
       </c>
     </row>
@@ -942,12 +958,22 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>backlog</t>
+          <t>doing</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>主権者</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-08-29 15:42</t>
+          <t>2026-08-29 16:48</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>下書き済(hackathon/agent_harness_20260829/docs/submission.md)。動画 URL を入れて送信</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
kanban: S07 硝子(Liquid Glass 風 UI)を Backlog に追加、発注書 step-07 と kanban.py add コマンド
Apple WWDC25 の Liquid Glass を参照し、StatusView / ApprovalView を glassEffect 化する
見た目だけの Step(macOS 26 API は #available で分岐、macOS 14 はフォールバック)。

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/kanban.xlsx
+++ b/docs/kanban.xlsx
@@ -483,7 +483,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Backlog (0)</t>
+          <t>Backlog (1)</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
@@ -503,11 +503,18 @@
       </c>
       <c r="F1" s="5" t="inlineStr">
         <is>
-          <t>updated 2026-08-29 16:48</t>
+          <t>updated 2026-08-29 19:28</t>
         </is>
       </c>
     </row>
     <row r="2" ht="58" customHeight="1">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>S07  硝子 Liquid Glass 風 UI(StatusView / ApprovalView を glassEffect 化)
+ · 2026-08-29 19:28
+Apple WWDC25 Liquid Glass 参照。見た目だけ、承認ロジック不変。Best UI 軸</t>
+        </is>
+      </c>
       <c r="B2" s="10" t="inlineStr">
         <is>
           <t>D01  デモ動画(3 分)・README 仕上げ
@@ -595,7 +602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -977,6 +984,39 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>S07</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>硝子 Liquid Glass 風 UI(StatusView / ApprovalView を glassEffect 化)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>docs/steps/step-07-glass-ui.md</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>backlog</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>2026-08-29 19:28</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Apple WWDC25 Liquid Glass 参照。見た目だけ、承認ロジック不変。Best UI 軸</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
kanban: S07〜S11 を Done(統合 PR #12 を main にマージ)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/kanban.xlsx
+++ b/docs/kanban.xlsx
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -493,17 +493,17 @@
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>Review(Qodo) (5)</t>
+          <t>Review(Qodo) (0)</t>
         </is>
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
-          <t>Done (7)</t>
+          <t>Done (12)</t>
         </is>
       </c>
       <c r="F1" s="5" t="inlineStr">
         <is>
-          <t>updated 2026-08-29 20:05</t>
+          <t>updated 2026-08-29 20:36</t>
         </is>
       </c>
     </row>
@@ -515,13 +515,6 @@
 主権者: docs/demo.md の台本で撮影(3 分)</t>
         </is>
       </c>
-      <c r="C2" s="8" t="inlineStr">
-        <is>
-          <t>S07  硝子 Liquid Glass 風 UI(StatusView / ApprovalView を glassEffect 化)
-agent · 2026-08-29 20:05
-全 UI(Status/Approval/HUD/Settings)をガラス化。統合 PR #12 で Qodo 待ち</t>
-        </is>
-      </c>
       <c r="D2" s="9" t="inlineStr">
         <is>
           <t>S00  骨組み(Package / .gitignore / Qodo / 発注書 / kanban)
@@ -538,13 +531,6 @@
 下書き済(hackathon/agent_harness_20260829/docs/submission.md)。動画 URL を入れて送信</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
-        <is>
-          <t>S08  焔(詠唱中に画面の縁を炎が囲う演出・設定で ON/OFF)
-agent · 2026-08-29 20:05
-統合 PR #12 に合流(#10 は close 可)</t>
-        </is>
-      </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
           <t>S01  ハーネス(TrueForge + OpenAI + Bright Data MCP + 呪文)
@@ -554,13 +540,6 @@
       </c>
     </row>
     <row r="4" ht="58" customHeight="1">
-      <c r="C4" s="8" t="inlineStr">
-        <is>
-          <t>S09  実機検証修正: ⌘長押し・HUD・キャンセル・⏎承認・設定・UI英語化・録音修正
- · 2026-08-29 20:05
-統合 PR #12 に合流(#11 は close 可)</t>
-        </is>
-      </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
           <t>S02  索敵・特定 `aishow scan`(ContextPack / detect)
@@ -570,13 +549,6 @@
       </c>
     </row>
     <row r="5" ht="58" customHeight="1">
-      <c r="C5" s="8" t="inlineStr">
-        <is>
-          <t>S10  権限の持続(自己署名で署名・make install 固定パス・許可ダイアログ自動表示・許可後に自動開始)
- · 2026-08-29 20:05
-PR #12</t>
-        </is>
-      </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
           <t>S03  発動 `aishow cast`(貼り付け・クリップボード復元)
@@ -586,13 +558,6 @@
       </c>
     </row>
     <row r="6" ht="58" customHeight="1">
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>S11  マイク選択設定(System default / 指定デバイス、AirPods HFP 劣化回避)
- · 2026-08-29 20:05
-PR #12。実機で AirPods 接続時の切替を確認したい</t>
-        </is>
-      </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
           <t>S04  詠唱 `aishow chant`(録音 → OpenAI STT)
@@ -616,6 +581,51 @@
           <t>S06  常駐 `Aishow.app`(メニューバー・ホットキー・承認 UI)
 agent · 2026-08-29 16:47
 PR #7 マージ(make app OK、常駐確認。GUI 通しは主権者が実施)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="58" customHeight="1">
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>S07  硝子 Liquid Glass 風 UI(StatusView / ApprovalView を glassEffect 化)
+agent · 2026-08-29 20:36
+PR #12 で main にマージ(1e86364)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="58" customHeight="1">
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>S08  焔(詠唱中に画面の縁を炎が囲う演出・設定で ON/OFF)
+agent · 2026-08-29 20:36
+PR #12 で main にマージ(1e86364)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="58" customHeight="1">
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>S09  実機検証修正: ⌘長押し・HUD・キャンセル・⏎承認・設定・UI英語化・録音修正
+ · 2026-08-29 20:36
+PR #12 で main にマージ(1e86364)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="58" customHeight="1">
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>S10  権限の持続(自己署名で署名・make install 固定パス・許可ダイアログ自動表示・許可後に自動開始)
+ · 2026-08-29 20:36
+PR #12 で main にマージ(1e86364)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="58" customHeight="1">
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>S11  マイク選択設定(System default / 指定デバイス、AirPods HFP 劣化回避)
+ · 2026-08-29 20:36
+録音は AVCaptureSession 化、Bluetooth 入力は内蔵マイクへ自動フォールバック</t>
         </is>
       </c>
     </row>
@@ -1030,7 +1040,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>done</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1040,12 +1050,12 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-08-29 20:05</t>
+          <t>2026-08-29 20:36</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>全 UI(Status/Approval/HUD/Settings)をガラス化。統合 PR #12 で Qodo 待ち</t>
+          <t>PR #12 で main にマージ(1e86364)</t>
         </is>
       </c>
     </row>
@@ -1067,7 +1077,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>done</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1077,12 +1087,12 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-08-29 20:05</t>
+          <t>2026-08-29 20:36</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>統合 PR #12 に合流(#10 は close 可)</t>
+          <t>PR #12 で main にマージ(1e86364)</t>
         </is>
       </c>
     </row>
@@ -1104,17 +1114,17 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>done</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-08-29 20:05</t>
+          <t>2026-08-29 20:36</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>統合 PR #12 に合流(#11 は close 可)</t>
+          <t>PR #12 で main にマージ(1e86364)</t>
         </is>
       </c>
     </row>
@@ -1136,17 +1146,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>done</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-08-29 20:05</t>
+          <t>2026-08-29 20:36</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>PR #12</t>
+          <t>PR #12 で main にマージ(1e86364)</t>
         </is>
       </c>
     </row>
@@ -1168,17 +1178,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>review</t>
+          <t>done</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-08-29 20:05</t>
+          <t>2026-08-29 20:36</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>PR #12。実機で AirPods 接続時の切替を確認したい</t>
+          <t>録音は AVCaptureSession 化、Bluetooth 入力は内蔵マイクへ自動フォールバック</t>
         </is>
       </c>
     </row>

</xml_diff>